<commit_message>
Added New File WriteDynamicDataInExcel.java
</commit_message>
<xml_diff>
--- a/resources/testdata.xlsx
+++ b/resources/testdata.xlsx
@@ -6,20 +6,46 @@
     <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet2" r:id="rId3" sheetId="1"/>
+    <sheet name="Sheet3" r:id="rId3" sheetId="1"/>
+    <sheet name="Sheet1" r:id="rId4" sheetId="2"/>
+    <sheet name="Sheet2" r:id="rId5" sheetId="3"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="30">
+  <si>
+    <t>Bowler</t>
+  </si>
+  <si>
+    <t>SkillSet</t>
+  </si>
+  <si>
+    <t>Bowling Hand</t>
+  </si>
+  <si>
+    <t>Bumrah</t>
+  </si>
+  <si>
+    <t>Yorker</t>
+  </si>
+  <si>
+    <t>Right</t>
+  </si>
+  <si>
+    <t>Boult</t>
+  </si>
+  <si>
+    <t>Swing</t>
+  </si>
+  <si>
+    <t>Left</t>
+  </si>
   <si>
     <t>Batter</t>
   </si>
   <si>
-    <t>Bowler</t>
-  </si>
-  <si>
     <t>All-Rounder</t>
   </si>
   <si>
@@ -35,9 +61,6 @@
     <t>Rohit</t>
   </si>
   <si>
-    <t>Bumrah</t>
-  </si>
-  <si>
     <t>Santner</t>
   </si>
   <si>
@@ -48,6 +71,39 @@
   </si>
   <si>
     <t>Krunal</t>
+  </si>
+  <si>
+    <t>james</t>
+  </si>
+  <si>
+    <t>steve</t>
+  </si>
+  <si>
+    <t>Smith</t>
+  </si>
+  <si>
+    <t>harry</t>
+  </si>
+  <si>
+    <t>brook</t>
+  </si>
+  <si>
+    <t>Aus</t>
+  </si>
+  <si>
+    <t>ENG</t>
+  </si>
+  <si>
+    <t>BAT</t>
+  </si>
+  <si>
+    <t>BOWL</t>
+  </si>
+  <si>
+    <t>TEST</t>
+  </si>
+  <si>
+    <t>ODI</t>
   </si>
 </sst>
 </file>
@@ -92,51 +148,200 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="0">
-        <v>1</v>
-      </c>
       <c r="C1" t="s" s="0">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
         <v>9</v>
       </c>
+      <c r="B1" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>16</v>
+      </c>
       <c r="B4" t="s" s="0">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>